<commit_message>
Update recessed top30 ecosystem summary to six-period total ranking
</commit_message>
<xml_diff>
--- a/recessed_top30_brand_ecosystem_summary.xlsx
+++ b/recessed_top30_brand_ecosystem_summary.xlsx
@@ -413,20 +413,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -442,45 +443,50 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>6期总销售额</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>方案判断</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>技术路线</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>主要生态系统</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>202504</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>202506</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>202508</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>202510</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>202511</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Last30days</t>
         </is>
@@ -495,37 +501,40 @@
           <t>Philips Hue</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" t="n">
+        <v>6825420</v>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>自研闭环生态</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Zigbee/Bridge/Matter过渡</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Hue App, Alexa, Google, Apple HomeKit, Siri</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>494117</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>1078450</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>984069</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>1417714</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>1569137</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>1281933</v>
       </c>
     </row>
@@ -538,37 +547,40 @@
           <t>Govee</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" t="n">
+        <v>2705206</v>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>自研闭环生态</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Wi‑Fi + Bluetooth + Matter</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Govee, Alexa, Google, Matter</t>
         </is>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>217884</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>292099</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>337415</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>591815</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>764520</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>501473</v>
       </c>
     </row>
@@ -581,37 +593,40 @@
           <t>SikSog</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" t="n">
+        <v>2275906</v>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>通用方案（证据弱，非自研倾向）</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Bluetooth为主</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Alexa</t>
         </is>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>154421</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>261462</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>361812</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>462383</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>652238</v>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>383590</v>
       </c>
     </row>
@@ -621,41 +636,44 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Lumary</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Tuya/Smart Life高相关</t>
-        </is>
+          <t>POWERASIA</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1864741</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Wi‑Fi + Bluetooth</t>
+          <t>Tuya Smart</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>Wi‑Fi/Hub混合</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>Alexa, Google, Siri</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>115229</v>
-      </c>
       <c r="G5" t="n">
-        <v>184071</v>
+        <v>306134</v>
       </c>
       <c r="H5" t="n">
-        <v>300031</v>
+        <v>364427</v>
       </c>
       <c r="I5" t="n">
-        <v>288641</v>
+        <v>261616</v>
       </c>
       <c r="J5" t="n">
-        <v>393490</v>
+        <v>388398</v>
       </c>
       <c r="K5" t="n">
-        <v>167537</v>
+        <v>389404</v>
+      </c>
+      <c r="L5" t="n">
+        <v>154762</v>
       </c>
     </row>
     <row r="6">
@@ -664,41 +682,44 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>POWERASIA</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Tuya Smart</t>
-        </is>
+          <t>Lumary</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1448999</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Wi‑Fi/Hub混合</t>
+          <t>Tuya/Smart Life高相关</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>Wi‑Fi + Bluetooth</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>Alexa, Google, Siri</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>306134</v>
-      </c>
       <c r="G6" t="n">
-        <v>364427</v>
+        <v>115229</v>
       </c>
       <c r="H6" t="n">
-        <v>261616</v>
+        <v>184071</v>
       </c>
       <c r="I6" t="n">
-        <v>388398</v>
+        <v>300031</v>
       </c>
       <c r="J6" t="n">
-        <v>389404</v>
+        <v>288641</v>
       </c>
       <c r="K6" t="n">
-        <v>154762</v>
+        <v>393490</v>
+      </c>
+      <c r="L6" t="n">
+        <v>167537</v>
       </c>
     </row>
     <row r="7">
@@ -707,41 +728,44 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ChangM</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>通用方案（非自研倾向）</t>
-        </is>
+          <t>CLOUDY BAY</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>863223</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Bluetooth/App</t>
+          <t>Smart Life/Tuya高相关</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Alexa, App</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>24920</v>
+          <t>Wi‑Fi</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Alexa, Google Home</t>
+        </is>
       </c>
       <c r="G7" t="n">
-        <v>44162</v>
+        <v>183013</v>
       </c>
       <c r="H7" t="n">
-        <v>58786</v>
+        <v>154286</v>
       </c>
       <c r="I7" t="n">
-        <v>78202</v>
+        <v>121782</v>
       </c>
       <c r="J7" t="n">
-        <v>87813</v>
+        <v>132827</v>
       </c>
       <c r="K7" t="n">
-        <v>121294</v>
+        <v>154734</v>
+      </c>
+      <c r="L7" t="n">
+        <v>116581</v>
       </c>
     </row>
     <row r="8">
@@ -753,37 +777,40 @@
           <t>Feit Electric</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" t="n">
+        <v>531831</v>
+      </c>
+      <c r="D8" t="inlineStr">
         <is>
           <t>Tuya高相关/自有前台App</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Wi‑Fi 2.4GHz</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Alexa, Google, Home Assistant(Tuya侧)</t>
         </is>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>1610</v>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>126344</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>102848</v>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>2375</v>
       </c>
-      <c r="J8" t="n">
+      <c r="K8" t="n">
         <v>177551</v>
       </c>
-      <c r="K8" t="n">
+      <c r="L8" t="n">
         <v>121103</v>
       </c>
     </row>
@@ -793,41 +820,44 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CLOUDY BAY</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Smart Life/Tuya高相关</t>
-        </is>
+          <t>YGS-Tech</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>511245</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>通用方案（Tuya待证）</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
           <t>Wi‑Fi</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Alexa, Google Home</t>
         </is>
       </c>
-      <c r="F9" t="n">
-        <v>183013</v>
-      </c>
       <c r="G9" t="n">
-        <v>154286</v>
+        <v>34473</v>
       </c>
       <c r="H9" t="n">
-        <v>121782</v>
+        <v>33798</v>
       </c>
       <c r="I9" t="n">
-        <v>132827</v>
+        <v>102216</v>
       </c>
       <c r="J9" t="n">
-        <v>154734</v>
+        <v>110490</v>
       </c>
       <c r="K9" t="n">
-        <v>116581</v>
+        <v>134782</v>
+      </c>
+      <c r="L9" t="n">
+        <v>95486</v>
       </c>
     </row>
     <row r="10">
@@ -836,41 +866,44 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>YGS-Tech</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>通用方案（Tuya待证）</t>
-        </is>
+          <t>Peteme</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>464676</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Wi‑Fi</t>
+          <t>通用方案（待证）</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Alexa, Google Home</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>34473</v>
+          <t>Wi‑Fi/Bluetooth待证</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Alexa/Google待证</t>
+        </is>
       </c>
       <c r="G10" t="n">
-        <v>33798</v>
+        <v>81206</v>
       </c>
       <c r="H10" t="n">
-        <v>102216</v>
+        <v>89475</v>
       </c>
       <c r="I10" t="n">
-        <v>110490</v>
+        <v>61107</v>
       </c>
       <c r="J10" t="n">
-        <v>134782</v>
+        <v>90156</v>
       </c>
       <c r="K10" t="n">
-        <v>95486</v>
+        <v>100587</v>
+      </c>
+      <c r="L10" t="n">
+        <v>42145</v>
       </c>
     </row>
     <row r="11">
@@ -879,41 +912,44 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>inShareplus</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>通用方案（Tuya待证）</t>
-        </is>
+          <t>ChangM</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>415177</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Wi‑Fi</t>
+          <t>通用方案（非自研倾向）</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Alexa, Google</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>51092</v>
+          <t>Bluetooth/App</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Alexa, App</t>
+        </is>
       </c>
       <c r="G11" t="n">
-        <v>67119</v>
+        <v>24920</v>
       </c>
       <c r="H11" t="n">
-        <v>63083</v>
+        <v>44162</v>
       </c>
       <c r="I11" t="n">
-        <v>68951</v>
+        <v>58786</v>
       </c>
       <c r="J11" t="n">
-        <v>77424</v>
+        <v>78202</v>
       </c>
       <c r="K11" t="n">
-        <v>62424</v>
+        <v>87813</v>
+      </c>
+      <c r="L11" t="n">
+        <v>121294</v>
       </c>
     </row>
     <row r="12">
@@ -922,41 +958,44 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SHUNLEE</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>通用方案（待证）</t>
-        </is>
+          <t>inShareplus</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>390093</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Wi‑Fi/Bluetooth待证</t>
+          <t>通用方案（Tuya待证）</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Alexa/Google待证</t>
-        </is>
-      </c>
-      <c r="F12" t="n">
-        <v>0</v>
+          <t>Wi‑Fi</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Alexa, Google</t>
+        </is>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>51092</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>67119</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>63083</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>68951</v>
       </c>
       <c r="K12" t="n">
-        <v>42576</v>
+        <v>77424</v>
+      </c>
+      <c r="L12" t="n">
+        <v>62424</v>
       </c>
     </row>
     <row r="13">
@@ -965,41 +1004,44 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Peteme</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>通用方案（待证）</t>
-        </is>
+          <t>Amico</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>260184</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Wi‑Fi/Bluetooth待证</t>
+          <t>传统照明品牌延伸/通用方案</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Alexa/Google待证</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>81206</v>
+          <t>路线待证</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>待证</t>
+        </is>
       </c>
       <c r="G13" t="n">
-        <v>89475</v>
+        <v>24946</v>
       </c>
       <c r="H13" t="n">
-        <v>61107</v>
+        <v>55324</v>
       </c>
       <c r="I13" t="n">
-        <v>90156</v>
+        <v>59003</v>
       </c>
       <c r="J13" t="n">
-        <v>100587</v>
+        <v>47444</v>
       </c>
       <c r="K13" t="n">
-        <v>42145</v>
+        <v>50426</v>
+      </c>
+      <c r="L13" t="n">
+        <v>23041</v>
       </c>
     </row>
     <row r="14">
@@ -1008,41 +1050,44 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DUSKTEC</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>通用方案（待证）</t>
-        </is>
+          <t>Sunco Lighting</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>198793</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Wi‑Fi/Bluetooth待证</t>
+          <t>传统照明品牌延伸</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Alexa/Google待证</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>0</v>
+          <t>路线待证</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>待证</t>
+        </is>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>16853</v>
       </c>
       <c r="H14" t="n">
-        <v>3987</v>
+        <v>25733</v>
       </c>
       <c r="I14" t="n">
-        <v>31039</v>
+        <v>44986</v>
       </c>
       <c r="J14" t="n">
-        <v>35027</v>
+        <v>41805</v>
       </c>
       <c r="K14" t="n">
-        <v>39386</v>
+        <v>40178</v>
+      </c>
+      <c r="L14" t="n">
+        <v>29238</v>
       </c>
     </row>
     <row r="15">
@@ -1054,37 +1099,40 @@
           <t>Cync</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" t="n">
+        <v>195204</v>
+      </c>
+      <c r="D15" t="inlineStr">
         <is>
           <t>GE/Cync自有生态</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>Wi‑Fi/Bluetooth/Matter侧</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Alexa, Google, Matter</t>
         </is>
       </c>
-      <c r="F15" t="n">
+      <c r="G15" t="n">
         <v>24280</v>
       </c>
-      <c r="G15" t="n">
+      <c r="H15" t="n">
         <v>25477</v>
       </c>
-      <c r="H15" t="n">
+      <c r="I15" t="n">
         <v>16166</v>
       </c>
-      <c r="I15" t="n">
+      <c r="J15" t="n">
         <v>39415</v>
       </c>
-      <c r="J15" t="n">
+      <c r="K15" t="n">
         <v>56553</v>
       </c>
-      <c r="K15" t="n">
+      <c r="L15" t="n">
         <v>33313</v>
       </c>
     </row>
@@ -1094,41 +1142,44 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ASD</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>通用照明品牌，智能边缘线</t>
-        </is>
+          <t>VARICART</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>134214</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>场景型智能灯，路线混合</t>
+          <t>通用方案（待证）</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
+          <t>路线待证</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
           <t>待证</t>
         </is>
       </c>
-      <c r="F16" t="n">
-        <v>10108</v>
-      </c>
       <c r="G16" t="n">
-        <v>3952</v>
+        <v>6780</v>
       </c>
       <c r="H16" t="n">
-        <v>3978</v>
+        <v>15338</v>
       </c>
       <c r="I16" t="n">
-        <v>20502</v>
+        <v>18718</v>
       </c>
       <c r="J16" t="n">
-        <v>18963</v>
+        <v>26919</v>
       </c>
       <c r="K16" t="n">
-        <v>31518</v>
+        <v>50435</v>
+      </c>
+      <c r="L16" t="n">
+        <v>16024</v>
       </c>
     </row>
     <row r="17">
@@ -1137,41 +1188,44 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sunco Lighting</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>传统照明品牌延伸</t>
-        </is>
+          <t>LightingWill</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>113547</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
+          <t>通用照明品牌/边缘智能</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
           <t>路线待证</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>待证</t>
         </is>
       </c>
-      <c r="F17" t="n">
-        <v>16853</v>
-      </c>
       <c r="G17" t="n">
-        <v>25733</v>
+        <v>22108</v>
       </c>
       <c r="H17" t="n">
-        <v>44986</v>
+        <v>20788</v>
       </c>
       <c r="I17" t="n">
-        <v>41805</v>
+        <v>13731</v>
       </c>
       <c r="J17" t="n">
-        <v>40178</v>
+        <v>21448</v>
       </c>
       <c r="K17" t="n">
-        <v>29238</v>
+        <v>23263</v>
+      </c>
+      <c r="L17" t="n">
+        <v>12209</v>
       </c>
     </row>
     <row r="18">
@@ -1180,26 +1234,26 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Lichaser</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
+          <t>DUSKTEC</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>109439</v>
+      </c>
+      <c r="D18" t="inlineStr">
         <is>
           <t>通用方案（待证）</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>Wi‑Fi/Bluetooth待证</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>Alexa/Google待证</t>
         </is>
-      </c>
-      <c r="F18" t="n">
-        <v>0</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
@@ -1208,13 +1262,16 @@
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>13342</v>
+        <v>3987</v>
       </c>
       <c r="J18" t="n">
-        <v>25208</v>
+        <v>31039</v>
       </c>
       <c r="K18" t="n">
-        <v>25876</v>
+        <v>35027</v>
+      </c>
+      <c r="L18" t="n">
+        <v>39386</v>
       </c>
     </row>
     <row r="19">
@@ -1223,41 +1280,44 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Amico</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>传统照明品牌延伸/通用方案</t>
-        </is>
+          <t>HYDONG</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>106987</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
+          <t>通用方案（待证）</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
           <t>路线待证</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>待证</t>
         </is>
       </c>
-      <c r="F19" t="n">
-        <v>24946</v>
-      </c>
       <c r="G19" t="n">
-        <v>55324</v>
+        <v>10649</v>
       </c>
       <c r="H19" t="n">
-        <v>59003</v>
+        <v>16798</v>
       </c>
       <c r="I19" t="n">
-        <v>47444</v>
+        <v>16735</v>
       </c>
       <c r="J19" t="n">
-        <v>50426</v>
+        <v>20183</v>
       </c>
       <c r="K19" t="n">
-        <v>23041</v>
+        <v>22474</v>
+      </c>
+      <c r="L19" t="n">
+        <v>20148</v>
       </c>
     </row>
     <row r="20">
@@ -1266,41 +1326,44 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>HALO</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>传统照明品牌延伸</t>
-        </is>
+          <t>JULLISON</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>100374</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
+          <t>通用方案（待证）</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
           <t>路线待证</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>待证</t>
         </is>
       </c>
-      <c r="F20" t="n">
-        <v>7338</v>
-      </c>
       <c r="G20" t="n">
-        <v>8419</v>
+        <v>13229</v>
       </c>
       <c r="H20" t="n">
-        <v>6336</v>
+        <v>15119</v>
       </c>
       <c r="I20" t="n">
-        <v>12964</v>
+        <v>15749</v>
       </c>
       <c r="J20" t="n">
-        <v>20912</v>
+        <v>20369</v>
       </c>
       <c r="K20" t="n">
-        <v>22102</v>
+        <v>20789</v>
+      </c>
+      <c r="L20" t="n">
+        <v>15119</v>
       </c>
     </row>
     <row r="21">
@@ -1309,41 +1372,44 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Lightdot</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>通用方案（待证）</t>
-        </is>
+          <t>Juno</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>90280</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>路线待证</t>
+          <t>待补证</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>待证</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>0</v>
+          <t>待补证</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>待补证</t>
+        </is>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>15587</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>16921</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>12418</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>22777</v>
       </c>
       <c r="K21" t="n">
-        <v>20198</v>
+        <v>17052</v>
+      </c>
+      <c r="L21" t="n">
+        <v>5525</v>
       </c>
     </row>
     <row r="22">
@@ -1352,41 +1418,44 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>HYDONG</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>通用方案（待证）</t>
-        </is>
+          <t>ASD</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>89021</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>路线待证</t>
+          <t>通用照明品牌，智能边缘线</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
+          <t>场景型智能灯，路线混合</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
           <t>待证</t>
         </is>
       </c>
-      <c r="F22" t="n">
-        <v>10649</v>
-      </c>
       <c r="G22" t="n">
-        <v>16798</v>
+        <v>10108</v>
       </c>
       <c r="H22" t="n">
-        <v>16735</v>
+        <v>3952</v>
       </c>
       <c r="I22" t="n">
-        <v>20183</v>
+        <v>3978</v>
       </c>
       <c r="J22" t="n">
-        <v>22474</v>
+        <v>20502</v>
       </c>
       <c r="K22" t="n">
-        <v>20148</v>
+        <v>18963</v>
+      </c>
+      <c r="L22" t="n">
+        <v>31518</v>
       </c>
     </row>
     <row r="23">
@@ -1395,41 +1464,44 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>HAMRVL</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>通用方案（待证）</t>
-        </is>
+          <t>HALO</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>78071</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
+          <t>传统照明品牌延伸</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
           <t>路线待证</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>待证</t>
         </is>
       </c>
-      <c r="F23" t="n">
-        <v>0</v>
-      </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>7338</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>8419</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>6336</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>12964</v>
       </c>
       <c r="K23" t="n">
-        <v>17196</v>
+        <v>20912</v>
+      </c>
+      <c r="L23" t="n">
+        <v>22102</v>
       </c>
     </row>
     <row r="24">
@@ -1438,41 +1510,44 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>VARICART</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>通用方案（待证）</t>
-        </is>
+          <t>Art3d</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>77110</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>路线待证</t>
+          <t>待补证</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>待证</t>
-        </is>
-      </c>
-      <c r="F24" t="n">
-        <v>6780</v>
+          <t>待补证</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>待补证</t>
+        </is>
       </c>
       <c r="G24" t="n">
-        <v>15338</v>
+        <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>18718</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>26919</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>50435</v>
+        <v>77110</v>
       </c>
       <c r="K24" t="n">
-        <v>16024</v>
+        <v>0</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -1481,41 +1556,44 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>JULLISON</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>通用方案（待证）</t>
-        </is>
+          <t>Aoketezm</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>75920</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>路线待证</t>
+          <t>待补证</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>待证</t>
-        </is>
-      </c>
-      <c r="F25" t="n">
-        <v>13229</v>
+          <t>待补证</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>待补证</t>
+        </is>
       </c>
       <c r="G25" t="n">
-        <v>15119</v>
+        <v>14167</v>
       </c>
       <c r="H25" t="n">
-        <v>15749</v>
+        <v>16256</v>
       </c>
       <c r="I25" t="n">
-        <v>20369</v>
+        <v>15382</v>
       </c>
       <c r="J25" t="n">
-        <v>20789</v>
+        <v>23447</v>
       </c>
       <c r="K25" t="n">
-        <v>15119</v>
+        <v>6668</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -1524,41 +1602,44 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>LEDLightsWorld</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
+          <t>Vanance</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>73605</v>
+      </c>
+      <c r="D26" t="inlineStr">
         <is>
           <t>通用方案（待证）</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>路线待证</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>待证</t>
         </is>
-      </c>
-      <c r="F26" t="n">
-        <v>0</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>10949</v>
+        <v>16319</v>
       </c>
       <c r="I26" t="n">
-        <v>16642</v>
+        <v>15639</v>
       </c>
       <c r="J26" t="n">
-        <v>17226</v>
+        <v>15469</v>
       </c>
       <c r="K26" t="n">
-        <v>14599</v>
+        <v>14449</v>
+      </c>
+      <c r="L26" t="n">
+        <v>11729</v>
       </c>
     </row>
     <row r="27">
@@ -1567,41 +1648,44 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>NeatiEase</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>通用方案（待证）</t>
-        </is>
+          <t>INFIBRITE</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>69105</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>路线待证</t>
+          <t>待补证</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>待证</t>
-        </is>
-      </c>
-      <c r="F27" t="n">
-        <v>0</v>
+          <t>待补证</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>待补证</t>
+        </is>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>24716</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>13200</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>10328</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>1039</v>
       </c>
       <c r="K27" t="n">
-        <v>14476</v>
+        <v>11918</v>
+      </c>
+      <c r="L27" t="n">
+        <v>7904</v>
       </c>
     </row>
     <row r="28">
@@ -1610,41 +1694,44 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Xskyㅤ</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>系统整合型品牌（非Tuya白牌心智）</t>
-        </is>
+          <t>Dcvoltfield</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>65256</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Zigbee 3.0 + Matter Bridge</t>
+          <t>待补证</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Alexa, Google, Siri/HomeKit, Home Assistant, SmartThings</t>
-        </is>
-      </c>
-      <c r="F28" t="n">
-        <v>8955</v>
+          <t>待补证</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>待补证</t>
+        </is>
       </c>
       <c r="G28" t="n">
-        <v>10410</v>
+        <v>4885</v>
       </c>
       <c r="H28" t="n">
-        <v>11798</v>
+        <v>9359</v>
       </c>
       <c r="I28" t="n">
-        <v>11306</v>
+        <v>12919</v>
       </c>
       <c r="J28" t="n">
-        <v>9702</v>
+        <v>13489</v>
       </c>
       <c r="K28" t="n">
-        <v>12315</v>
+        <v>14245</v>
+      </c>
+      <c r="L28" t="n">
+        <v>10359</v>
       </c>
     </row>
     <row r="29">
@@ -1653,41 +1740,44 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>LightingWill</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>通用照明品牌/边缘智能</t>
-        </is>
+          <t>Xskyㅤ</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>64486</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>路线待证</t>
+          <t>系统整合型品牌（非Tuya白牌心智）</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>待证</t>
-        </is>
-      </c>
-      <c r="F29" t="n">
-        <v>22108</v>
+          <t>Zigbee 3.0 + Matter Bridge</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Alexa, Google, Siri/HomeKit, Home Assistant, SmartThings</t>
+        </is>
       </c>
       <c r="G29" t="n">
-        <v>20788</v>
+        <v>8955</v>
       </c>
       <c r="H29" t="n">
-        <v>13731</v>
+        <v>10410</v>
       </c>
       <c r="I29" t="n">
-        <v>21448</v>
+        <v>11798</v>
       </c>
       <c r="J29" t="n">
-        <v>23263</v>
+        <v>11306</v>
       </c>
       <c r="K29" t="n">
-        <v>12209</v>
+        <v>9702</v>
+      </c>
+      <c r="L29" t="n">
+        <v>12315</v>
       </c>
     </row>
     <row r="30">
@@ -1696,26 +1786,26 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>DeerTalk</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
+          <t>Lichaser</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>64426</v>
+      </c>
+      <c r="D30" t="inlineStr">
         <is>
           <t>通用方案（待证）</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>路线待证</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>待证</t>
         </is>
-      </c>
-      <c r="F30" t="n">
-        <v>0</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
@@ -1724,13 +1814,16 @@
         <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>8596</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>14101</v>
+        <v>13342</v>
       </c>
       <c r="K30" t="n">
-        <v>11879</v>
+        <v>25208</v>
+      </c>
+      <c r="L30" t="n">
+        <v>25876</v>
       </c>
     </row>
     <row r="31">
@@ -1739,41 +1832,44 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Vanance</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
+          <t>LEDLightsWorld</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>59416</v>
+      </c>
+      <c r="D31" t="inlineStr">
         <is>
           <t>通用方案（待证）</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>路线待证</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>待证</t>
         </is>
       </c>
-      <c r="F31" t="n">
+      <c r="G31" t="n">
         <v>0</v>
       </c>
-      <c r="G31" t="n">
-        <v>16319</v>
-      </c>
       <c r="H31" t="n">
-        <v>15639</v>
+        <v>0</v>
       </c>
       <c r="I31" t="n">
-        <v>15469</v>
+        <v>10949</v>
       </c>
       <c r="J31" t="n">
-        <v>14449</v>
+        <v>16642</v>
       </c>
       <c r="K31" t="n">
-        <v>11729</v>
+        <v>17226</v>
+      </c>
+      <c r="L31" t="n">
+        <v>14599</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix top30 ecosystem summary to show six-period total clearly
</commit_message>
<xml_diff>
--- a/recessed_top30_brand_ecosystem_summary.xlsx
+++ b/recessed_top30_brand_ecosystem_summary.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="check" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -416,18 +417,18 @@
   <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -448,47 +449,47 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>202506</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>202508</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>202510</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>202511</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Last30days</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>方案判断</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>技术路线</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>主要生态系统</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>202504</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>202506</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>202508</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>202510</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>202511</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Last30days</t>
         </is>
       </c>
     </row>
@@ -504,38 +505,38 @@
       <c r="C2" t="n">
         <v>6825420</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="n">
+        <v>494117</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1078450</v>
+      </c>
+      <c r="F2" t="n">
+        <v>984069</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1417714</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1569137</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1281933</v>
+      </c>
+      <c r="J2" t="inlineStr">
         <is>
           <t>自研闭环生态</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Zigbee/Bridge/Matter过渡</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Hue App, Alexa, Google, Apple HomeKit, Siri</t>
         </is>
-      </c>
-      <c r="G2" t="n">
-        <v>494117</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1078450</v>
-      </c>
-      <c r="I2" t="n">
-        <v>984069</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1417714</v>
-      </c>
-      <c r="K2" t="n">
-        <v>1569137</v>
-      </c>
-      <c r="L2" t="n">
-        <v>1281933</v>
       </c>
     </row>
     <row r="3">
@@ -550,38 +551,38 @@
       <c r="C3" t="n">
         <v>2705206</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" t="n">
+        <v>217884</v>
+      </c>
+      <c r="E3" t="n">
+        <v>292099</v>
+      </c>
+      <c r="F3" t="n">
+        <v>337415</v>
+      </c>
+      <c r="G3" t="n">
+        <v>591815</v>
+      </c>
+      <c r="H3" t="n">
+        <v>764520</v>
+      </c>
+      <c r="I3" t="n">
+        <v>501473</v>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>自研闭环生态</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Wi‑Fi + Bluetooth + Matter</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Govee, Alexa, Google, Matter</t>
         </is>
-      </c>
-      <c r="G3" t="n">
-        <v>217884</v>
-      </c>
-      <c r="H3" t="n">
-        <v>292099</v>
-      </c>
-      <c r="I3" t="n">
-        <v>337415</v>
-      </c>
-      <c r="J3" t="n">
-        <v>591815</v>
-      </c>
-      <c r="K3" t="n">
-        <v>764520</v>
-      </c>
-      <c r="L3" t="n">
-        <v>501473</v>
       </c>
     </row>
     <row r="4">
@@ -596,38 +597,38 @@
       <c r="C4" t="n">
         <v>2275906</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" t="n">
+        <v>154421</v>
+      </c>
+      <c r="E4" t="n">
+        <v>261462</v>
+      </c>
+      <c r="F4" t="n">
+        <v>361812</v>
+      </c>
+      <c r="G4" t="n">
+        <v>462383</v>
+      </c>
+      <c r="H4" t="n">
+        <v>652238</v>
+      </c>
+      <c r="I4" t="n">
+        <v>383590</v>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>通用方案（证据弱，非自研倾向）</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Bluetooth为主</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Alexa</t>
         </is>
-      </c>
-      <c r="G4" t="n">
-        <v>154421</v>
-      </c>
-      <c r="H4" t="n">
-        <v>261462</v>
-      </c>
-      <c r="I4" t="n">
-        <v>361812</v>
-      </c>
-      <c r="J4" t="n">
-        <v>462383</v>
-      </c>
-      <c r="K4" t="n">
-        <v>652238</v>
-      </c>
-      <c r="L4" t="n">
-        <v>383590</v>
       </c>
     </row>
     <row r="5">
@@ -642,38 +643,38 @@
       <c r="C5" t="n">
         <v>1864741</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" t="n">
+        <v>306134</v>
+      </c>
+      <c r="E5" t="n">
+        <v>364427</v>
+      </c>
+      <c r="F5" t="n">
+        <v>261616</v>
+      </c>
+      <c r="G5" t="n">
+        <v>388398</v>
+      </c>
+      <c r="H5" t="n">
+        <v>389404</v>
+      </c>
+      <c r="I5" t="n">
+        <v>154762</v>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>Tuya Smart</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Wi‑Fi/Hub混合</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Alexa, Google, Siri</t>
         </is>
-      </c>
-      <c r="G5" t="n">
-        <v>306134</v>
-      </c>
-      <c r="H5" t="n">
-        <v>364427</v>
-      </c>
-      <c r="I5" t="n">
-        <v>261616</v>
-      </c>
-      <c r="J5" t="n">
-        <v>388398</v>
-      </c>
-      <c r="K5" t="n">
-        <v>389404</v>
-      </c>
-      <c r="L5" t="n">
-        <v>154762</v>
       </c>
     </row>
     <row r="6">
@@ -688,38 +689,38 @@
       <c r="C6" t="n">
         <v>1448999</v>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" t="n">
+        <v>115229</v>
+      </c>
+      <c r="E6" t="n">
+        <v>184071</v>
+      </c>
+      <c r="F6" t="n">
+        <v>300031</v>
+      </c>
+      <c r="G6" t="n">
+        <v>288641</v>
+      </c>
+      <c r="H6" t="n">
+        <v>393490</v>
+      </c>
+      <c r="I6" t="n">
+        <v>167537</v>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>Tuya/Smart Life高相关</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Wi‑Fi + Bluetooth</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Alexa, Google, Siri</t>
         </is>
-      </c>
-      <c r="G6" t="n">
-        <v>115229</v>
-      </c>
-      <c r="H6" t="n">
-        <v>184071</v>
-      </c>
-      <c r="I6" t="n">
-        <v>300031</v>
-      </c>
-      <c r="J6" t="n">
-        <v>288641</v>
-      </c>
-      <c r="K6" t="n">
-        <v>393490</v>
-      </c>
-      <c r="L6" t="n">
-        <v>167537</v>
       </c>
     </row>
     <row r="7">
@@ -734,38 +735,38 @@
       <c r="C7" t="n">
         <v>863223</v>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" t="n">
+        <v>183013</v>
+      </c>
+      <c r="E7" t="n">
+        <v>154286</v>
+      </c>
+      <c r="F7" t="n">
+        <v>121782</v>
+      </c>
+      <c r="G7" t="n">
+        <v>132827</v>
+      </c>
+      <c r="H7" t="n">
+        <v>154734</v>
+      </c>
+      <c r="I7" t="n">
+        <v>116581</v>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>Smart Life/Tuya高相关</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>Wi‑Fi</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Alexa, Google Home</t>
         </is>
-      </c>
-      <c r="G7" t="n">
-        <v>183013</v>
-      </c>
-      <c r="H7" t="n">
-        <v>154286</v>
-      </c>
-      <c r="I7" t="n">
-        <v>121782</v>
-      </c>
-      <c r="J7" t="n">
-        <v>132827</v>
-      </c>
-      <c r="K7" t="n">
-        <v>154734</v>
-      </c>
-      <c r="L7" t="n">
-        <v>116581</v>
       </c>
     </row>
     <row r="8">
@@ -780,38 +781,38 @@
       <c r="C8" t="n">
         <v>531831</v>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" t="n">
+        <v>1610</v>
+      </c>
+      <c r="E8" t="n">
+        <v>126344</v>
+      </c>
+      <c r="F8" t="n">
+        <v>102848</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2375</v>
+      </c>
+      <c r="H8" t="n">
+        <v>177551</v>
+      </c>
+      <c r="I8" t="n">
+        <v>121103</v>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>Tuya高相关/自有前台App</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Wi‑Fi 2.4GHz</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>Alexa, Google, Home Assistant(Tuya侧)</t>
         </is>
-      </c>
-      <c r="G8" t="n">
-        <v>1610</v>
-      </c>
-      <c r="H8" t="n">
-        <v>126344</v>
-      </c>
-      <c r="I8" t="n">
-        <v>102848</v>
-      </c>
-      <c r="J8" t="n">
-        <v>2375</v>
-      </c>
-      <c r="K8" t="n">
-        <v>177551</v>
-      </c>
-      <c r="L8" t="n">
-        <v>121103</v>
       </c>
     </row>
     <row r="9">
@@ -826,38 +827,38 @@
       <c r="C9" t="n">
         <v>511245</v>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" t="n">
+        <v>34473</v>
+      </c>
+      <c r="E9" t="n">
+        <v>33798</v>
+      </c>
+      <c r="F9" t="n">
+        <v>102216</v>
+      </c>
+      <c r="G9" t="n">
+        <v>110490</v>
+      </c>
+      <c r="H9" t="n">
+        <v>134782</v>
+      </c>
+      <c r="I9" t="n">
+        <v>95486</v>
+      </c>
+      <c r="J9" t="inlineStr">
         <is>
           <t>通用方案（Tuya待证）</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>Wi‑Fi</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>Alexa, Google Home</t>
         </is>
-      </c>
-      <c r="G9" t="n">
-        <v>34473</v>
-      </c>
-      <c r="H9" t="n">
-        <v>33798</v>
-      </c>
-      <c r="I9" t="n">
-        <v>102216</v>
-      </c>
-      <c r="J9" t="n">
-        <v>110490</v>
-      </c>
-      <c r="K9" t="n">
-        <v>134782</v>
-      </c>
-      <c r="L9" t="n">
-        <v>95486</v>
       </c>
     </row>
     <row r="10">
@@ -872,38 +873,38 @@
       <c r="C10" t="n">
         <v>464676</v>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" t="n">
+        <v>81206</v>
+      </c>
+      <c r="E10" t="n">
+        <v>89475</v>
+      </c>
+      <c r="F10" t="n">
+        <v>61107</v>
+      </c>
+      <c r="G10" t="n">
+        <v>90156</v>
+      </c>
+      <c r="H10" t="n">
+        <v>100587</v>
+      </c>
+      <c r="I10" t="n">
+        <v>42145</v>
+      </c>
+      <c r="J10" t="inlineStr">
         <is>
           <t>通用方案（待证）</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Wi‑Fi/Bluetooth待证</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>Alexa/Google待证</t>
         </is>
-      </c>
-      <c r="G10" t="n">
-        <v>81206</v>
-      </c>
-      <c r="H10" t="n">
-        <v>89475</v>
-      </c>
-      <c r="I10" t="n">
-        <v>61107</v>
-      </c>
-      <c r="J10" t="n">
-        <v>90156</v>
-      </c>
-      <c r="K10" t="n">
-        <v>100587</v>
-      </c>
-      <c r="L10" t="n">
-        <v>42145</v>
       </c>
     </row>
     <row r="11">
@@ -918,38 +919,38 @@
       <c r="C11" t="n">
         <v>415177</v>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" t="n">
+        <v>24920</v>
+      </c>
+      <c r="E11" t="n">
+        <v>44162</v>
+      </c>
+      <c r="F11" t="n">
+        <v>58786</v>
+      </c>
+      <c r="G11" t="n">
+        <v>78202</v>
+      </c>
+      <c r="H11" t="n">
+        <v>87813</v>
+      </c>
+      <c r="I11" t="n">
+        <v>121294</v>
+      </c>
+      <c r="J11" t="inlineStr">
         <is>
           <t>通用方案（非自研倾向）</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>Bluetooth/App</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>Alexa, App</t>
         </is>
-      </c>
-      <c r="G11" t="n">
-        <v>24920</v>
-      </c>
-      <c r="H11" t="n">
-        <v>44162</v>
-      </c>
-      <c r="I11" t="n">
-        <v>58786</v>
-      </c>
-      <c r="J11" t="n">
-        <v>78202</v>
-      </c>
-      <c r="K11" t="n">
-        <v>87813</v>
-      </c>
-      <c r="L11" t="n">
-        <v>121294</v>
       </c>
     </row>
     <row r="12">
@@ -964,38 +965,38 @@
       <c r="C12" t="n">
         <v>390093</v>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" t="n">
+        <v>51092</v>
+      </c>
+      <c r="E12" t="n">
+        <v>67119</v>
+      </c>
+      <c r="F12" t="n">
+        <v>63083</v>
+      </c>
+      <c r="G12" t="n">
+        <v>68951</v>
+      </c>
+      <c r="H12" t="n">
+        <v>77424</v>
+      </c>
+      <c r="I12" t="n">
+        <v>62424</v>
+      </c>
+      <c r="J12" t="inlineStr">
         <is>
           <t>通用方案（Tuya待证）</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>Wi‑Fi</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>Alexa, Google</t>
         </is>
-      </c>
-      <c r="G12" t="n">
-        <v>51092</v>
-      </c>
-      <c r="H12" t="n">
-        <v>67119</v>
-      </c>
-      <c r="I12" t="n">
-        <v>63083</v>
-      </c>
-      <c r="J12" t="n">
-        <v>68951</v>
-      </c>
-      <c r="K12" t="n">
-        <v>77424</v>
-      </c>
-      <c r="L12" t="n">
-        <v>62424</v>
       </c>
     </row>
     <row r="13">
@@ -1010,38 +1011,38 @@
       <c r="C13" t="n">
         <v>260184</v>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" t="n">
+        <v>24946</v>
+      </c>
+      <c r="E13" t="n">
+        <v>55324</v>
+      </c>
+      <c r="F13" t="n">
+        <v>59003</v>
+      </c>
+      <c r="G13" t="n">
+        <v>47444</v>
+      </c>
+      <c r="H13" t="n">
+        <v>50426</v>
+      </c>
+      <c r="I13" t="n">
+        <v>23041</v>
+      </c>
+      <c r="J13" t="inlineStr">
         <is>
           <t>传统照明品牌延伸/通用方案</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>路线待证</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>待证</t>
         </is>
-      </c>
-      <c r="G13" t="n">
-        <v>24946</v>
-      </c>
-      <c r="H13" t="n">
-        <v>55324</v>
-      </c>
-      <c r="I13" t="n">
-        <v>59003</v>
-      </c>
-      <c r="J13" t="n">
-        <v>47444</v>
-      </c>
-      <c r="K13" t="n">
-        <v>50426</v>
-      </c>
-      <c r="L13" t="n">
-        <v>23041</v>
       </c>
     </row>
     <row r="14">
@@ -1056,38 +1057,38 @@
       <c r="C14" t="n">
         <v>198793</v>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" t="n">
+        <v>16853</v>
+      </c>
+      <c r="E14" t="n">
+        <v>25733</v>
+      </c>
+      <c r="F14" t="n">
+        <v>44986</v>
+      </c>
+      <c r="G14" t="n">
+        <v>41805</v>
+      </c>
+      <c r="H14" t="n">
+        <v>40178</v>
+      </c>
+      <c r="I14" t="n">
+        <v>29238</v>
+      </c>
+      <c r="J14" t="inlineStr">
         <is>
           <t>传统照明品牌延伸</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>路线待证</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>待证</t>
         </is>
-      </c>
-      <c r="G14" t="n">
-        <v>16853</v>
-      </c>
-      <c r="H14" t="n">
-        <v>25733</v>
-      </c>
-      <c r="I14" t="n">
-        <v>44986</v>
-      </c>
-      <c r="J14" t="n">
-        <v>41805</v>
-      </c>
-      <c r="K14" t="n">
-        <v>40178</v>
-      </c>
-      <c r="L14" t="n">
-        <v>29238</v>
       </c>
     </row>
     <row r="15">
@@ -1102,38 +1103,38 @@
       <c r="C15" t="n">
         <v>195204</v>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" t="n">
+        <v>24280</v>
+      </c>
+      <c r="E15" t="n">
+        <v>25477</v>
+      </c>
+      <c r="F15" t="n">
+        <v>16166</v>
+      </c>
+      <c r="G15" t="n">
+        <v>39415</v>
+      </c>
+      <c r="H15" t="n">
+        <v>56553</v>
+      </c>
+      <c r="I15" t="n">
+        <v>33313</v>
+      </c>
+      <c r="J15" t="inlineStr">
         <is>
           <t>GE/Cync自有生态</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>Wi‑Fi/Bluetooth/Matter侧</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>Alexa, Google, Matter</t>
         </is>
-      </c>
-      <c r="G15" t="n">
-        <v>24280</v>
-      </c>
-      <c r="H15" t="n">
-        <v>25477</v>
-      </c>
-      <c r="I15" t="n">
-        <v>16166</v>
-      </c>
-      <c r="J15" t="n">
-        <v>39415</v>
-      </c>
-      <c r="K15" t="n">
-        <v>56553</v>
-      </c>
-      <c r="L15" t="n">
-        <v>33313</v>
       </c>
     </row>
     <row r="16">
@@ -1148,38 +1149,38 @@
       <c r="C16" t="n">
         <v>134214</v>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" t="n">
+        <v>6780</v>
+      </c>
+      <c r="E16" t="n">
+        <v>15338</v>
+      </c>
+      <c r="F16" t="n">
+        <v>18718</v>
+      </c>
+      <c r="G16" t="n">
+        <v>26919</v>
+      </c>
+      <c r="H16" t="n">
+        <v>50435</v>
+      </c>
+      <c r="I16" t="n">
+        <v>16024</v>
+      </c>
+      <c r="J16" t="inlineStr">
         <is>
           <t>通用方案（待证）</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>路线待证</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>待证</t>
         </is>
-      </c>
-      <c r="G16" t="n">
-        <v>6780</v>
-      </c>
-      <c r="H16" t="n">
-        <v>15338</v>
-      </c>
-      <c r="I16" t="n">
-        <v>18718</v>
-      </c>
-      <c r="J16" t="n">
-        <v>26919</v>
-      </c>
-      <c r="K16" t="n">
-        <v>50435</v>
-      </c>
-      <c r="L16" t="n">
-        <v>16024</v>
       </c>
     </row>
     <row r="17">
@@ -1194,38 +1195,38 @@
       <c r="C17" t="n">
         <v>113547</v>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" t="n">
+        <v>22108</v>
+      </c>
+      <c r="E17" t="n">
+        <v>20788</v>
+      </c>
+      <c r="F17" t="n">
+        <v>13731</v>
+      </c>
+      <c r="G17" t="n">
+        <v>21448</v>
+      </c>
+      <c r="H17" t="n">
+        <v>23263</v>
+      </c>
+      <c r="I17" t="n">
+        <v>12209</v>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>通用照明品牌/边缘智能</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>路线待证</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>待证</t>
         </is>
-      </c>
-      <c r="G17" t="n">
-        <v>22108</v>
-      </c>
-      <c r="H17" t="n">
-        <v>20788</v>
-      </c>
-      <c r="I17" t="n">
-        <v>13731</v>
-      </c>
-      <c r="J17" t="n">
-        <v>21448</v>
-      </c>
-      <c r="K17" t="n">
-        <v>23263</v>
-      </c>
-      <c r="L17" t="n">
-        <v>12209</v>
       </c>
     </row>
     <row r="18">
@@ -1240,38 +1241,38 @@
       <c r="C18" t="n">
         <v>109439</v>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>3987</v>
+      </c>
+      <c r="G18" t="n">
+        <v>31039</v>
+      </c>
+      <c r="H18" t="n">
+        <v>35027</v>
+      </c>
+      <c r="I18" t="n">
+        <v>39386</v>
+      </c>
+      <c r="J18" t="inlineStr">
         <is>
           <t>通用方案（待证）</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>Wi‑Fi/Bluetooth待证</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>Alexa/Google待证</t>
         </is>
-      </c>
-      <c r="G18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" t="n">
-        <v>3987</v>
-      </c>
-      <c r="J18" t="n">
-        <v>31039</v>
-      </c>
-      <c r="K18" t="n">
-        <v>35027</v>
-      </c>
-      <c r="L18" t="n">
-        <v>39386</v>
       </c>
     </row>
     <row r="19">
@@ -1286,38 +1287,38 @@
       <c r="C19" t="n">
         <v>106987</v>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" t="n">
+        <v>10649</v>
+      </c>
+      <c r="E19" t="n">
+        <v>16798</v>
+      </c>
+      <c r="F19" t="n">
+        <v>16735</v>
+      </c>
+      <c r="G19" t="n">
+        <v>20183</v>
+      </c>
+      <c r="H19" t="n">
+        <v>22474</v>
+      </c>
+      <c r="I19" t="n">
+        <v>20148</v>
+      </c>
+      <c r="J19" t="inlineStr">
         <is>
           <t>通用方案（待证）</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>路线待证</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>待证</t>
         </is>
-      </c>
-      <c r="G19" t="n">
-        <v>10649</v>
-      </c>
-      <c r="H19" t="n">
-        <v>16798</v>
-      </c>
-      <c r="I19" t="n">
-        <v>16735</v>
-      </c>
-      <c r="J19" t="n">
-        <v>20183</v>
-      </c>
-      <c r="K19" t="n">
-        <v>22474</v>
-      </c>
-      <c r="L19" t="n">
-        <v>20148</v>
       </c>
     </row>
     <row r="20">
@@ -1332,38 +1333,38 @@
       <c r="C20" t="n">
         <v>100374</v>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" t="n">
+        <v>13229</v>
+      </c>
+      <c r="E20" t="n">
+        <v>15119</v>
+      </c>
+      <c r="F20" t="n">
+        <v>15749</v>
+      </c>
+      <c r="G20" t="n">
+        <v>20369</v>
+      </c>
+      <c r="H20" t="n">
+        <v>20789</v>
+      </c>
+      <c r="I20" t="n">
+        <v>15119</v>
+      </c>
+      <c r="J20" t="inlineStr">
         <is>
           <t>通用方案（待证）</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>路线待证</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>待证</t>
         </is>
-      </c>
-      <c r="G20" t="n">
-        <v>13229</v>
-      </c>
-      <c r="H20" t="n">
-        <v>15119</v>
-      </c>
-      <c r="I20" t="n">
-        <v>15749</v>
-      </c>
-      <c r="J20" t="n">
-        <v>20369</v>
-      </c>
-      <c r="K20" t="n">
-        <v>20789</v>
-      </c>
-      <c r="L20" t="n">
-        <v>15119</v>
       </c>
     </row>
     <row r="21">
@@ -1378,38 +1379,38 @@
       <c r="C21" t="n">
         <v>90280</v>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" t="n">
+        <v>15587</v>
+      </c>
+      <c r="E21" t="n">
+        <v>16921</v>
+      </c>
+      <c r="F21" t="n">
+        <v>12418</v>
+      </c>
+      <c r="G21" t="n">
+        <v>22777</v>
+      </c>
+      <c r="H21" t="n">
+        <v>17052</v>
+      </c>
+      <c r="I21" t="n">
+        <v>5525</v>
+      </c>
+      <c r="J21" t="inlineStr">
         <is>
           <t>待补证</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>待补证</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>待补证</t>
         </is>
-      </c>
-      <c r="G21" t="n">
-        <v>15587</v>
-      </c>
-      <c r="H21" t="n">
-        <v>16921</v>
-      </c>
-      <c r="I21" t="n">
-        <v>12418</v>
-      </c>
-      <c r="J21" t="n">
-        <v>22777</v>
-      </c>
-      <c r="K21" t="n">
-        <v>17052</v>
-      </c>
-      <c r="L21" t="n">
-        <v>5525</v>
       </c>
     </row>
     <row r="22">
@@ -1424,38 +1425,38 @@
       <c r="C22" t="n">
         <v>89021</v>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" t="n">
+        <v>10108</v>
+      </c>
+      <c r="E22" t="n">
+        <v>3952</v>
+      </c>
+      <c r="F22" t="n">
+        <v>3978</v>
+      </c>
+      <c r="G22" t="n">
+        <v>20502</v>
+      </c>
+      <c r="H22" t="n">
+        <v>18963</v>
+      </c>
+      <c r="I22" t="n">
+        <v>31518</v>
+      </c>
+      <c r="J22" t="inlineStr">
         <is>
           <t>通用照明品牌，智能边缘线</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>场景型智能灯，路线混合</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>待证</t>
         </is>
-      </c>
-      <c r="G22" t="n">
-        <v>10108</v>
-      </c>
-      <c r="H22" t="n">
-        <v>3952</v>
-      </c>
-      <c r="I22" t="n">
-        <v>3978</v>
-      </c>
-      <c r="J22" t="n">
-        <v>20502</v>
-      </c>
-      <c r="K22" t="n">
-        <v>18963</v>
-      </c>
-      <c r="L22" t="n">
-        <v>31518</v>
       </c>
     </row>
     <row r="23">
@@ -1470,38 +1471,38 @@
       <c r="C23" t="n">
         <v>78071</v>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" t="n">
+        <v>7338</v>
+      </c>
+      <c r="E23" t="n">
+        <v>8419</v>
+      </c>
+      <c r="F23" t="n">
+        <v>6336</v>
+      </c>
+      <c r="G23" t="n">
+        <v>12964</v>
+      </c>
+      <c r="H23" t="n">
+        <v>20912</v>
+      </c>
+      <c r="I23" t="n">
+        <v>22102</v>
+      </c>
+      <c r="J23" t="inlineStr">
         <is>
           <t>传统照明品牌延伸</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>路线待证</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>待证</t>
         </is>
-      </c>
-      <c r="G23" t="n">
-        <v>7338</v>
-      </c>
-      <c r="H23" t="n">
-        <v>8419</v>
-      </c>
-      <c r="I23" t="n">
-        <v>6336</v>
-      </c>
-      <c r="J23" t="n">
-        <v>12964</v>
-      </c>
-      <c r="K23" t="n">
-        <v>20912</v>
-      </c>
-      <c r="L23" t="n">
-        <v>22102</v>
       </c>
     </row>
     <row r="24">
@@ -1516,23 +1517,17 @@
       <c r="C24" t="n">
         <v>77110</v>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>待补证</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>待补证</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>待补证</t>
-        </is>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>77110</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -1540,14 +1535,20 @@
       <c r="I24" t="n">
         <v>0</v>
       </c>
-      <c r="J24" t="n">
-        <v>77110</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>待补证</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>待补证</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>待补证</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -1562,38 +1563,38 @@
       <c r="C25" t="n">
         <v>75920</v>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" t="n">
+        <v>14167</v>
+      </c>
+      <c r="E25" t="n">
+        <v>16256</v>
+      </c>
+      <c r="F25" t="n">
+        <v>15382</v>
+      </c>
+      <c r="G25" t="n">
+        <v>23447</v>
+      </c>
+      <c r="H25" t="n">
+        <v>6668</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="inlineStr">
         <is>
           <t>待补证</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>待补证</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>待补证</t>
         </is>
-      </c>
-      <c r="G25" t="n">
-        <v>14167</v>
-      </c>
-      <c r="H25" t="n">
-        <v>16256</v>
-      </c>
-      <c r="I25" t="n">
-        <v>15382</v>
-      </c>
-      <c r="J25" t="n">
-        <v>23447</v>
-      </c>
-      <c r="K25" t="n">
-        <v>6668</v>
-      </c>
-      <c r="L25" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -1608,38 +1609,38 @@
       <c r="C26" t="n">
         <v>73605</v>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>16319</v>
+      </c>
+      <c r="F26" t="n">
+        <v>15639</v>
+      </c>
+      <c r="G26" t="n">
+        <v>15469</v>
+      </c>
+      <c r="H26" t="n">
+        <v>14449</v>
+      </c>
+      <c r="I26" t="n">
+        <v>11729</v>
+      </c>
+      <c r="J26" t="inlineStr">
         <is>
           <t>通用方案（待证）</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>路线待证</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>待证</t>
         </is>
-      </c>
-      <c r="G26" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" t="n">
-        <v>16319</v>
-      </c>
-      <c r="I26" t="n">
-        <v>15639</v>
-      </c>
-      <c r="J26" t="n">
-        <v>15469</v>
-      </c>
-      <c r="K26" t="n">
-        <v>14449</v>
-      </c>
-      <c r="L26" t="n">
-        <v>11729</v>
       </c>
     </row>
     <row r="27">
@@ -1654,38 +1655,38 @@
       <c r="C27" t="n">
         <v>69105</v>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" t="n">
+        <v>24716</v>
+      </c>
+      <c r="E27" t="n">
+        <v>13200</v>
+      </c>
+      <c r="F27" t="n">
+        <v>10328</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1039</v>
+      </c>
+      <c r="H27" t="n">
+        <v>11918</v>
+      </c>
+      <c r="I27" t="n">
+        <v>7904</v>
+      </c>
+      <c r="J27" t="inlineStr">
         <is>
           <t>待补证</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>待补证</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>待补证</t>
         </is>
-      </c>
-      <c r="G27" t="n">
-        <v>24716</v>
-      </c>
-      <c r="H27" t="n">
-        <v>13200</v>
-      </c>
-      <c r="I27" t="n">
-        <v>10328</v>
-      </c>
-      <c r="J27" t="n">
-        <v>1039</v>
-      </c>
-      <c r="K27" t="n">
-        <v>11918</v>
-      </c>
-      <c r="L27" t="n">
-        <v>7904</v>
       </c>
     </row>
     <row r="28">
@@ -1700,38 +1701,38 @@
       <c r="C28" t="n">
         <v>65256</v>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" t="n">
+        <v>4885</v>
+      </c>
+      <c r="E28" t="n">
+        <v>9359</v>
+      </c>
+      <c r="F28" t="n">
+        <v>12919</v>
+      </c>
+      <c r="G28" t="n">
+        <v>13489</v>
+      </c>
+      <c r="H28" t="n">
+        <v>14245</v>
+      </c>
+      <c r="I28" t="n">
+        <v>10359</v>
+      </c>
+      <c r="J28" t="inlineStr">
         <is>
           <t>待补证</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>待补证</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>待补证</t>
         </is>
-      </c>
-      <c r="G28" t="n">
-        <v>4885</v>
-      </c>
-      <c r="H28" t="n">
-        <v>9359</v>
-      </c>
-      <c r="I28" t="n">
-        <v>12919</v>
-      </c>
-      <c r="J28" t="n">
-        <v>13489</v>
-      </c>
-      <c r="K28" t="n">
-        <v>14245</v>
-      </c>
-      <c r="L28" t="n">
-        <v>10359</v>
       </c>
     </row>
     <row r="29">
@@ -1746,38 +1747,38 @@
       <c r="C29" t="n">
         <v>64486</v>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" t="n">
+        <v>8955</v>
+      </c>
+      <c r="E29" t="n">
+        <v>10410</v>
+      </c>
+      <c r="F29" t="n">
+        <v>11798</v>
+      </c>
+      <c r="G29" t="n">
+        <v>11306</v>
+      </c>
+      <c r="H29" t="n">
+        <v>9702</v>
+      </c>
+      <c r="I29" t="n">
+        <v>12315</v>
+      </c>
+      <c r="J29" t="inlineStr">
         <is>
           <t>系统整合型品牌（非Tuya白牌心智）</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>Zigbee 3.0 + Matter Bridge</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>Alexa, Google, Siri/HomeKit, Home Assistant, SmartThings</t>
         </is>
-      </c>
-      <c r="G29" t="n">
-        <v>8955</v>
-      </c>
-      <c r="H29" t="n">
-        <v>10410</v>
-      </c>
-      <c r="I29" t="n">
-        <v>11798</v>
-      </c>
-      <c r="J29" t="n">
-        <v>11306</v>
-      </c>
-      <c r="K29" t="n">
-        <v>9702</v>
-      </c>
-      <c r="L29" t="n">
-        <v>12315</v>
       </c>
     </row>
     <row r="30">
@@ -1792,38 +1793,38 @@
       <c r="C30" t="n">
         <v>64426</v>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
+        <v>13342</v>
+      </c>
+      <c r="H30" t="n">
+        <v>25208</v>
+      </c>
+      <c r="I30" t="n">
+        <v>25876</v>
+      </c>
+      <c r="J30" t="inlineStr">
         <is>
           <t>通用方案（待证）</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>路线待证</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>待证</t>
         </is>
-      </c>
-      <c r="G30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" t="n">
-        <v>13342</v>
-      </c>
-      <c r="K30" t="n">
-        <v>25208</v>
-      </c>
-      <c r="L30" t="n">
-        <v>25876</v>
       </c>
     </row>
     <row r="31">
@@ -1838,38 +1839,64 @@
       <c r="C31" t="n">
         <v>59416</v>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>10949</v>
+      </c>
+      <c r="G31" t="n">
+        <v>16642</v>
+      </c>
+      <c r="H31" t="n">
+        <v>17226</v>
+      </c>
+      <c r="I31" t="n">
+        <v>14599</v>
+      </c>
+      <c r="J31" t="inlineStr">
         <is>
           <t>通用方案（待证）</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>路线待证</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>待证</t>
         </is>
       </c>
-      <c r="G31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" t="n">
-        <v>10949</v>
-      </c>
-      <c r="J31" t="n">
-        <v>16642</v>
-      </c>
-      <c r="K31" t="n">
-        <v>17226</v>
-      </c>
-      <c r="L31" t="n">
-        <v>14599</v>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>本表按6期总销售额排序，第三列就是6期总销售额</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update top30 ecosystem summary with evidence notes
</commit_message>
<xml_diff>
--- a/recessed_top30_brand_ecosystem_summary.xlsx
+++ b/recessed_top30_brand_ecosystem_summary.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:M31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -429,6 +429,7 @@
     <col width="30" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
     <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="38" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -492,6 +493,11 @@
           <t>主要生态系统</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>证据/判断依据</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -538,6 +544,11 @@
           <t>Hue App, Alexa, Google, Apple HomeKit, Siri</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>标题+官网/公开资料强证据</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -584,6 +595,11 @@
           <t>Govee, Alexa, Google, Matter</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>标题强证据</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -617,7 +633,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>通用方案（证据弱，非自研倾向）</t>
+          <t>通用方案，非自研倾向</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -628,6 +644,11 @@
       <c r="L4" t="inlineStr">
         <is>
           <t>Alexa</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>标题信号：Bluetooth Control + Alexa，公开品牌生态弱</t>
         </is>
       </c>
     </row>
@@ -676,6 +697,11 @@
           <t>Alexa, Google, Siri</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>品牌页明确写 TuYa Smart App</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -722,6 +748,11 @@
           <t>Alexa, Google, Siri</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>外部社区有 Lumary(Tuya)/Local Tuya 证据</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -768,6 +799,11 @@
           <t>Alexa, Google Home</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>社区出现 Smart Life 关联</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -814,6 +850,11 @@
           <t>Alexa, Google, Home Assistant(Tuya侧)</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Home Assistant / Tuya 社区证据</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -847,7 +888,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>通用方案（Tuya待证）</t>
+          <t>通用方案，非自研倾向</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -858,6 +899,11 @@
       <c r="L9" t="inlineStr">
         <is>
           <t>Alexa, Google Home</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>标题信号：WiFi + Alexa/Google Home</t>
         </is>
       </c>
     </row>
@@ -893,17 +939,22 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>通用方案（待证）</t>
+          <t>通用方案，非自研倾向</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Wi‑Fi/Bluetooth待证</t>
+          <t>Wi‑Fi/Bluetooth可能并存</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Alexa/Google待证</t>
+          <t>Alexa/Google（按标题信号）</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>公开证据弱，按同类 listing 标题信号判断</t>
         </is>
       </c>
     </row>
@@ -939,7 +990,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>通用方案（非自研倾向）</t>
+          <t>通用方案，非自研倾向</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -950,6 +1001,11 @@
       <c r="L11" t="inlineStr">
         <is>
           <t>Alexa, App</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>标题信号：Bluetooth/App/Alexa，公开系统证据弱</t>
         </is>
       </c>
     </row>
@@ -985,7 +1041,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>通用方案（Tuya待证）</t>
+          <t>通用方案，非自研倾向</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -996,6 +1052,11 @@
       <c r="L12" t="inlineStr">
         <is>
           <t>Alexa, Google</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>标题信号：WiFi + Alexa/Google</t>
         </is>
       </c>
     </row>
@@ -1031,17 +1092,22 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>传统照明品牌延伸/通用方案</t>
+          <t>传统照明延伸，智能线偏通用方案</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>路线待证</t>
+          <t>路线公开证据弱</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>待证</t>
+          <t>生态公开证据弱</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>公开证据弱，按品牌定位判断</t>
         </is>
       </c>
     </row>
@@ -1077,17 +1143,22 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>传统照明品牌延伸</t>
+          <t>自有前台App + Smart Life/Tuya兼容</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>路线待证</t>
+          <t>Wi‑Fi</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>待证</t>
+          <t>Sunco Smart Lighting, Alexa, Google</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Sunco 官方博客明确写 Sunco app，也可用 Smart Life/Tuya</t>
         </is>
       </c>
     </row>
@@ -1136,6 +1207,11 @@
           <t>Alexa, Google, Matter</t>
         </is>
       </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>品牌生态公开明确</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1169,17 +1245,22 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>通用方案（待证）</t>
+          <t>通用方案，非自研倾向</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>路线待证</t>
+          <t>路线公开证据弱</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>待证</t>
+          <t>Alexa/Google（按标题信号）</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>公开证据弱，按标题信号判断</t>
         </is>
       </c>
     </row>
@@ -1220,12 +1301,17 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>路线待证</t>
+          <t>路线公开证据弱</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>待证</t>
+          <t>Alexa/Google（按标题信号）</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>公开证据弱，按标题信号判断</t>
         </is>
       </c>
     </row>
@@ -1261,17 +1347,22 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>通用方案（待证）</t>
+          <t>通用方案，BRmesh系控制</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Wi‑Fi/Bluetooth待证</t>
+          <t>Bluetooth Mesh / App</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Alexa/Google待证</t>
+          <t>Alexa, Google, Siri</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>manuals.plus 指向 BRmesh app；标题写 Alexa/Siri/Google</t>
         </is>
       </c>
     </row>
@@ -1307,17 +1398,22 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>通用方案（待证）</t>
+          <t>通用方案，非自研倾向</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>路线待证</t>
+          <t>路线公开证据弱</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>待证</t>
+          <t>Alexa/Google（按标题信号）</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>公开证据弱，按标题信号判断</t>
         </is>
       </c>
     </row>
@@ -1353,17 +1449,22 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>通用方案（待证）</t>
+          <t>通用方案，非自研倾向</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>路线待证</t>
+          <t>路线公开证据弱</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>待证</t>
+          <t>Alexa/Google（按标题信号）</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>公开证据弱，按标题信号判断</t>
         </is>
       </c>
     </row>
@@ -1399,17 +1500,22 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>待补证</t>
+          <t>公开证据弱，按标题信号判断</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>待补证</t>
+          <t>路线公开证据弱</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>待补证</t>
+          <t>生态公开证据弱</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>公开证据不足</t>
         </is>
       </c>
     </row>
@@ -1445,17 +1551,22 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>通用照明品牌，智能边缘线</t>
+          <t>自有前台App + 通用连接层</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>场景型智能灯，路线混合</t>
+          <t>Wi‑Fi + Bluetooth</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>待证</t>
+          <t>ASD Smart App, Alexa, Google</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>外部页面明确写 ASD SMART APP + Alexa/Google</t>
         </is>
       </c>
     </row>
@@ -1496,12 +1607,17 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>路线待证</t>
+          <t>路线公开证据弱</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>待证</t>
+          <t>生态公开证据弱</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>公开证据弱，按品牌定位判断</t>
         </is>
       </c>
     </row>
@@ -1537,17 +1653,22 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>待补证</t>
+          <t>公开证据弱，按标题信号判断</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>待补证</t>
+          <t>路线公开证据弱</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>待补证</t>
+          <t>生态公开证据弱</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>公开证据不足</t>
         </is>
       </c>
     </row>
@@ -1583,17 +1704,22 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>待补证</t>
+          <t>公开证据弱，按标题信号判断</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>待补证</t>
+          <t>路线公开证据弱</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>待补证</t>
+          <t>生态公开证据弱</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>公开证据不足</t>
         </is>
       </c>
     </row>
@@ -1629,17 +1755,22 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>通用方案（待证）</t>
+          <t>通用方案，非自研倾向</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>路线待证</t>
+          <t>路线公开证据弱</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>待证</t>
+          <t>Alexa/Google（按标题信号）</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>公开证据弱，按标题信号判断</t>
         </is>
       </c>
     </row>
@@ -1675,17 +1806,22 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>待补证</t>
+          <t>公开证据弱，按标题信号判断</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>待补证</t>
+          <t>路线公开证据弱</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>待补证</t>
+          <t>生态公开证据弱</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>公开证据不足</t>
         </is>
       </c>
     </row>
@@ -1721,17 +1857,22 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>待补证</t>
+          <t>公开证据弱，按标题信号判断</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>待补证</t>
+          <t>路线公开证据弱</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>待补证</t>
+          <t>生态公开证据弱</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>公开证据不足</t>
         </is>
       </c>
     </row>
@@ -1780,6 +1921,11 @@
           <t>Alexa, Google, Siri/HomeKit, Home Assistant, SmartThings</t>
         </is>
       </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>官网+Amazon标题+社区信号</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1813,17 +1959,22 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>通用方案（待证）</t>
+          <t>通用方案，非自研倾向</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>路线待证</t>
+          <t>Wi‑Fi/Bluetooth待定</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>待证</t>
+          <t>Alexa/Google（按标题信号）</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>公开证据弱，按标题与同类品牌信号判断</t>
         </is>
       </c>
     </row>
@@ -1859,17 +2010,22 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>通用方案（待证）</t>
+          <t>通用方案，非自研倾向</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>路线待证</t>
+          <t>路线公开证据弱</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>待证</t>
+          <t>Alexa/Google（按标题信号）</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>公开证据弱，按标题信号判断</t>
         </is>
       </c>
     </row>
@@ -1895,7 +2051,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>本表按6期总销售额排序，第三列就是6期总销售额</t>
+          <t>已尽量补齐公开证据；搜不到硬证据的品牌，改为“公开证据弱，按标题信号判断”，不再留“待证”空白。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Exclude decorative recessed kit noise from dedup outputs and summary
</commit_message>
<xml_diff>
--- a/recessed_top30_brand_ecosystem_summary.xlsx
+++ b/recessed_top30_brand_ecosystem_summary.xlsx
@@ -1627,26 +1627,26 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Art3d</t>
+          <t>Aoketezm</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>77110</v>
+        <v>75920</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>14167</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>16256</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>15382</v>
       </c>
       <c r="G24" t="n">
-        <v>77110</v>
+        <v>23447</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>6668</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
@@ -1678,48 +1678,48 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Aoketezm</t>
+          <t>Vanance</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>75920</v>
+        <v>73605</v>
       </c>
       <c r="D25" t="n">
-        <v>14167</v>
+        <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>16256</v>
+        <v>16319</v>
       </c>
       <c r="F25" t="n">
-        <v>15382</v>
+        <v>15639</v>
       </c>
       <c r="G25" t="n">
-        <v>23447</v>
+        <v>15469</v>
       </c>
       <c r="H25" t="n">
-        <v>6668</v>
+        <v>14449</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>11729</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
+          <t>通用方案，非自研倾向</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>路线公开证据弱</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Alexa/Google（按标题信号）</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
           <t>公开证据弱，按标题信号判断</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>路线公开证据弱</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>生态公开证据弱</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>公开证据不足</t>
         </is>
       </c>
     </row>
@@ -1729,33 +1729,33 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Vanance</t>
+          <t>INFIBRITE</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>73605</v>
+        <v>69105</v>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>24716</v>
       </c>
       <c r="E26" t="n">
-        <v>16319</v>
+        <v>13200</v>
       </c>
       <c r="F26" t="n">
-        <v>15639</v>
+        <v>10328</v>
       </c>
       <c r="G26" t="n">
-        <v>15469</v>
+        <v>1039</v>
       </c>
       <c r="H26" t="n">
-        <v>14449</v>
+        <v>11918</v>
       </c>
       <c r="I26" t="n">
-        <v>11729</v>
+        <v>7904</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>通用方案，非自研倾向</t>
+          <t>公开证据弱，按标题信号判断</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -1765,12 +1765,12 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Alexa/Google（按标题信号）</t>
+          <t>生态公开证据弱</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>公开证据弱，按标题信号判断</t>
+          <t>公开证据不足</t>
         </is>
       </c>
     </row>
@@ -1780,29 +1780,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>INFIBRITE</t>
+          <t>Dcvoltfield</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>69105</v>
+        <v>65256</v>
       </c>
       <c r="D27" t="n">
-        <v>24716</v>
+        <v>4885</v>
       </c>
       <c r="E27" t="n">
-        <v>13200</v>
+        <v>9359</v>
       </c>
       <c r="F27" t="n">
-        <v>10328</v>
+        <v>12919</v>
       </c>
       <c r="G27" t="n">
-        <v>1039</v>
+        <v>13489</v>
       </c>
       <c r="H27" t="n">
-        <v>11918</v>
+        <v>14245</v>
       </c>
       <c r="I27" t="n">
-        <v>7904</v>
+        <v>10359</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -1831,48 +1831,48 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Dcvoltfield</t>
+          <t>Xskyㅤ</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>65256</v>
+        <v>64486</v>
       </c>
       <c r="D28" t="n">
-        <v>4885</v>
+        <v>8955</v>
       </c>
       <c r="E28" t="n">
-        <v>9359</v>
+        <v>10410</v>
       </c>
       <c r="F28" t="n">
-        <v>12919</v>
+        <v>11798</v>
       </c>
       <c r="G28" t="n">
-        <v>13489</v>
+        <v>11306</v>
       </c>
       <c r="H28" t="n">
-        <v>14245</v>
+        <v>9702</v>
       </c>
       <c r="I28" t="n">
-        <v>10359</v>
+        <v>12315</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>公开证据弱，按标题信号判断</t>
+          <t>系统整合型品牌（非Tuya白牌心智）</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>路线公开证据弱</t>
+          <t>Zigbee 3.0 + Matter Bridge</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>生态公开证据弱</t>
+          <t>Alexa, Google, Siri/HomeKit, Home Assistant, SmartThings</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>公开证据不足</t>
+          <t>官网+Amazon标题+社区信号</t>
         </is>
       </c>
     </row>
@@ -1882,48 +1882,48 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Xskyㅤ</t>
+          <t>LEDLightsWorld</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>64486</v>
+        <v>59416</v>
       </c>
       <c r="D29" t="n">
-        <v>8955</v>
+        <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>10410</v>
+        <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>11798</v>
+        <v>10949</v>
       </c>
       <c r="G29" t="n">
-        <v>11306</v>
+        <v>16642</v>
       </c>
       <c r="H29" t="n">
-        <v>9702</v>
+        <v>17226</v>
       </c>
       <c r="I29" t="n">
-        <v>12315</v>
+        <v>14599</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>系统整合型品牌（非Tuya白牌心智）</t>
+          <t>通用方案，非自研倾向</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Zigbee 3.0 + Matter Bridge</t>
+          <t>路线公开证据弱</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Alexa, Google, Siri/HomeKit, Home Assistant, SmartThings</t>
+          <t>Alexa/Google（按标题信号）</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>官网+Amazon标题+社区信号</t>
+          <t>公开证据弱，按标题信号判断</t>
         </is>
       </c>
     </row>
@@ -1933,48 +1933,48 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Lichaser</t>
+          <t>Neliwo</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>64426</v>
+        <v>57969</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
       </c>
       <c r="E30" t="n">
-        <v>0</v>
+        <v>2799</v>
       </c>
       <c r="F30" t="n">
-        <v>0</v>
+        <v>3342</v>
       </c>
       <c r="G30" t="n">
-        <v>13342</v>
+        <v>22056</v>
       </c>
       <c r="H30" t="n">
-        <v>25208</v>
+        <v>19173</v>
       </c>
       <c r="I30" t="n">
-        <v>25876</v>
+        <v>10599</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>通用方案，非自研倾向</t>
+          <t>公开证据弱，按标题信号判断</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Wi‑Fi/Bluetooth待定</t>
+          <t>路线公开证据弱</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Alexa/Google（按标题信号）</t>
+          <t>生态公开证据弱</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>公开证据弱，按标题与同类品牌信号判断</t>
+          <t>公开证据不足</t>
         </is>
       </c>
     </row>
@@ -1984,33 +1984,33 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>LEDLightsWorld</t>
+          <t>CycevSun</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>59416</v>
+        <v>57754</v>
       </c>
       <c r="D31" t="n">
+        <v>16085</v>
+      </c>
+      <c r="E31" t="n">
+        <v>21322</v>
+      </c>
+      <c r="F31" t="n">
+        <v>9109</v>
+      </c>
+      <c r="G31" t="n">
+        <v>8269</v>
+      </c>
+      <c r="H31" t="n">
+        <v>2969</v>
+      </c>
+      <c r="I31" t="n">
         <v>0</v>
       </c>
-      <c r="E31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" t="n">
-        <v>10949</v>
-      </c>
-      <c r="G31" t="n">
-        <v>16642</v>
-      </c>
-      <c r="H31" t="n">
-        <v>17226</v>
-      </c>
-      <c r="I31" t="n">
-        <v>14599</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>通用方案，非自研倾向</t>
+          <t>公开证据弱，按标题信号判断</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2020,12 +2020,12 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Alexa/Google（按标题信号）</t>
+          <t>生态公开证据弱</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>公开证据弱，按标题信号判断</t>
+          <t>公开证据不足</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>已尽量补齐公开证据；搜不到硬证据的品牌，改为“公开证据弱，按标题信号判断”，不再留“待证”空白。</t>
+          <t>已排除 medicine cabinet / bathroom mirror / bulb / self-adhesive wall-panel kit 等非目标池内容。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add proof status to recessed top30 ecosystem summary
</commit_message>
<xml_diff>
--- a/recessed_top30_brand_ecosystem_summary.xlsx
+++ b/recessed_top30_brand_ecosystem_summary.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M31"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -426,10 +426,11 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
-    <col width="32" customWidth="1" min="12" max="12"/>
-    <col width="38" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -480,20 +481,25 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>证明状态</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>方案判断</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>技术路线</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>主要生态系统</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>证据/判断依据</t>
         </is>
@@ -531,20 +537,25 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
+          <t>已证明</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>自研闭环生态</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Zigbee/Bridge/Matter过渡</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Hue App, Alexa, Google, Apple HomeKit, Siri</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>标题+官网/公开资料强证据</t>
         </is>
@@ -582,22 +593,27 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
+          <t>已证明</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
           <t>自研闭环生态</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Wi‑Fi + Bluetooth + Matter</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Govee, Alexa, Google, Matter</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>标题强证据</t>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>标题+品牌公开资料强证据</t>
         </is>
       </c>
     </row>
@@ -633,22 +649,27 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>通用方案，非自研倾向</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Bluetooth为主</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Alexa</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>标题信号：Bluetooth Control + Alexa，公开品牌生态弱</t>
+          <t>无法证明方案详情</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>持续搜索后未获足够公开硬证据</t>
         </is>
       </c>
     </row>
@@ -684,20 +705,25 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
+          <t>已证明</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
           <t>Tuya Smart</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Wi‑Fi/Hub混合</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Alexa, Google, Siri</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>品牌页明确写 TuYa Smart App</t>
         </is>
@@ -735,22 +761,27 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
+          <t>高相关推断</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
           <t>Tuya/Smart Life高相关</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Wi‑Fi + Bluetooth</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Alexa, Google, Siri</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>外部社区有 Lumary(Tuya)/Local Tuya 证据</t>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>外部社区有 Lumary(Tuya)/Local Tuya 证据，但非官方直接完整声明</t>
         </is>
       </c>
     </row>
@@ -786,22 +817,27 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
+          <t>高相关推断</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
           <t>Smart Life/Tuya高相关</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Wi‑Fi</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Alexa, Google Home</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>社区出现 Smart Life 关联</t>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>社区出现 Smart Life 关联，但官方直接证据不足</t>
         </is>
       </c>
     </row>
@@ -837,22 +873,27 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
+          <t>高相关推断</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
           <t>Tuya高相关/自有前台App</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>Wi‑Fi 2.4GHz</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>Alexa, Google, Home Assistant(Tuya侧)</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>Home Assistant / Tuya 社区证据</t>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Home Assistant / Tuya 社区证据强，但方案归属非官方完全直述</t>
         </is>
       </c>
     </row>
@@ -888,22 +929,27 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>通用方案，非自研倾向</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Wi‑Fi</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Alexa, Google Home</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>标题信号：WiFi + Alexa/Google Home</t>
+          <t>无法证明方案详情</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>持续搜索后未获足够公开硬证据</t>
         </is>
       </c>
     </row>
@@ -939,22 +985,27 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>通用方案，非自研倾向</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Wi‑Fi/Bluetooth可能并存</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Alexa/Google（按标题信号）</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>公开证据弱，按同类 listing 标题信号判断</t>
+          <t>无法证明方案详情</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>持续搜索后未获足够公开硬证据</t>
         </is>
       </c>
     </row>
@@ -990,22 +1041,27 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>通用方案，非自研倾向</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Bluetooth/App</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Alexa, App</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>标题信号：Bluetooth/App/Alexa，公开系统证据弱</t>
+          <t>无法证明方案详情</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>持续搜索后未获足够公开硬证据</t>
         </is>
       </c>
     </row>
@@ -1041,22 +1097,27 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>通用方案，非自研倾向</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Wi‑Fi</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Alexa, Google</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>标题信号：WiFi + Alexa/Google</t>
+          <t>无法证明方案详情</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>持续搜索后未获足够公开硬证据</t>
         </is>
       </c>
     </row>
@@ -1092,22 +1153,27 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>传统照明延伸，智能线偏通用方案</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>路线公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>生态公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>公开证据弱，按品牌定位判断</t>
+          <t>无法证明方案详情</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>持续搜索后未获足够公开硬证据</t>
         </is>
       </c>
     </row>
@@ -1143,20 +1209,25 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>自有前台App + Smart Life/Tuya兼容</t>
+          <t>已证明</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
+          <t>Sunco app + Smart Life/Tuya兼容</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
           <t>Wi‑Fi</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>Sunco Smart Lighting, Alexa, Google</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>Sunco 官方博客明确写 Sunco app，也可用 Smart Life/Tuya</t>
         </is>
@@ -1194,20 +1265,25 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
+          <t>已证明</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
           <t>GE/Cync自有生态</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>Wi‑Fi/Bluetooth/Matter侧</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>Alexa, Google, Matter</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>品牌生态公开明确</t>
         </is>
@@ -1245,22 +1321,27 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>通用方案，非自研倾向</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>路线公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Alexa/Google（按标题信号）</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>公开证据弱，按标题信号判断</t>
+          <t>无法证明方案详情</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>持续搜索后未获足够公开硬证据</t>
         </is>
       </c>
     </row>
@@ -1296,22 +1377,27 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>通用照明品牌/边缘智能</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>路线公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Alexa/Google（按标题信号）</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>公开证据弱，按标题信号判断</t>
+          <t>无法证明方案详情</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>持续搜索后未获足够公开硬证据</t>
         </is>
       </c>
     </row>
@@ -1347,22 +1433,27 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>通用方案，BRmesh系控制</t>
+          <t>已证明</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
+          <t>BRmesh系控制</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
           <t>Bluetooth Mesh / App</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>Alexa, Google, Siri</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>manuals.plus 指向 BRmesh app；标题写 Alexa/Siri/Google</t>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>说明书/手册公开写 BRmesh，标题写 Alexa/Siri/Google</t>
         </is>
       </c>
     </row>
@@ -1398,22 +1489,27 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>通用方案，非自研倾向</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>路线公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Alexa/Google（按标题信号）</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>公开证据弱，按标题信号判断</t>
+          <t>无法证明方案详情</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>持续搜索后未获足够公开硬证据</t>
         </is>
       </c>
     </row>
@@ -1449,22 +1545,27 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>通用方案，非自研倾向</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>路线公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Alexa/Google（按标题信号）</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>公开证据弱，按标题信号判断</t>
+          <t>无法证明方案详情</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>持续搜索后未获足够公开硬证据</t>
         </is>
       </c>
     </row>
@@ -1500,22 +1601,27 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>公开证据弱，按标题信号判断</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>路线公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>生态公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>公开证据不足</t>
+          <t>无法证明方案详情</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>未找到足够公开证据</t>
         </is>
       </c>
     </row>
@@ -1551,20 +1657,25 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>自有前台App + 通用连接层</t>
+          <t>已证明</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
+          <t>ASD SMART APP + 通用连接层</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
           <t>Wi‑Fi + Bluetooth</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>ASD Smart App, Alexa, Google</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>外部页面明确写 ASD SMART APP + Alexa/Google</t>
         </is>
@@ -1602,22 +1713,27 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>传统照明品牌延伸</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>路线公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>生态公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>公开证据弱，按品牌定位判断</t>
+          <t>无法证明方案详情</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>持续搜索后未获足够公开硬证据</t>
         </is>
       </c>
     </row>
@@ -1653,22 +1769,27 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>公开证据弱，按标题信号判断</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>路线公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>生态公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>公开证据不足</t>
+          <t>无法证明方案详情</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>未找到足够公开证据</t>
         </is>
       </c>
     </row>
@@ -1704,22 +1825,27 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>通用方案，非自研倾向</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>路线公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Alexa/Google（按标题信号）</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>公开证据弱，按标题信号判断</t>
+          <t>无法证明方案详情</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>持续搜索后未获足够公开硬证据</t>
         </is>
       </c>
     </row>
@@ -1755,22 +1881,27 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>公开证据弱，按标题信号判断</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>路线公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>生态公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>公开证据不足</t>
+          <t>无法证明方案详情</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>未找到足够公开证据</t>
         </is>
       </c>
     </row>
@@ -1806,22 +1937,27 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>公开证据弱，按标题信号判断</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>路线公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>生态公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>公开证据不足</t>
+          <t>无法证明方案详情</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>未找到足够公开证据</t>
         </is>
       </c>
     </row>
@@ -1857,20 +1993,25 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
+          <t>已证明</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
           <t>系统整合型品牌（非Tuya白牌心智）</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>Zigbee 3.0 + Matter Bridge</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>Alexa, Google, Siri/HomeKit, Home Assistant, SmartThings</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="N28" t="inlineStr">
         <is>
           <t>官网+Amazon标题+社区信号</t>
         </is>
@@ -1908,22 +2049,27 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>通用方案，非自研倾向</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>路线公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Alexa/Google（按标题信号）</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>公开证据弱，按标题信号判断</t>
+          <t>无法证明方案详情</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>持续搜索后未获足够公开硬证据</t>
         </is>
       </c>
     </row>
@@ -1959,22 +2105,27 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>公开证据弱，按标题信号判断</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>路线公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>生态公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>公开证据不足</t>
+          <t>无法证明方案详情</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>未找到足够公开证据</t>
         </is>
       </c>
     </row>
@@ -2010,22 +2161,27 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>公开证据弱，按标题信号判断</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>路线公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>生态公开证据弱</t>
+          <t>无法证明方案详情</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>公开证据不足</t>
+          <t>无法证明方案详情</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>未找到足够公开证据</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2051,7 +2207,19 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>已排除 medicine cabinet / bathroom mirror / bulb / self-adhesive wall-panel kit 等非目标池内容。</t>
+          <t>证明状态只保留三种：已证明 / 高相关推断 / 无法证明方案详情</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>规则</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>对持续搜索后仍无硬证据的品牌，直接写“无法证明方案详情”，不再用“待证/证据弱”</t>
         </is>
       </c>
     </row>

</xml_diff>